<commit_message>
chore: update bulk upload option of product
</commit_message>
<xml_diff>
--- a/public/templates/products_list_template.xlsx
+++ b/public/templates/products_list_template.xlsx
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t xml:space="preserve">slug</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -101,8 +98,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -298,18 +299,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" s="0" t="s">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>